<commit_message>
The reinforce agent is modified to weigh the entropy of the whole batch rather than the topk. Results seem to be more consistent. The CRN topology diversity graph is introduced.
</commit_message>
<xml_diff>
--- a/apps/RPA_3species_5rxns_REINFORCE/RPA_3species_5rxns_MAK_REINFORCE.xlsx
+++ b/apps/RPA_3species_5rxns_REINFORCE/RPA_3species_5rxns_MAK_REINFORCE.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="99">
   <si>
     <t>Timestamp</t>
   </si>
@@ -67,6 +67,12 @@
     <t>2025-11-03 15:22:05</t>
   </si>
   <si>
+    <t>2025-11-07 12:20:24</t>
+  </si>
+  <si>
+    <t>2025-11-07 15:10:13</t>
+  </si>
+  <si>
     <t>URL</t>
   </si>
   <si>
@@ -118,6 +124,12 @@
     <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/08537c0627b6441fb9ed6f6328eb2627</t>
   </si>
   <si>
+    <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/cb4a2ecf6dc447df8caee14bdedbe11e</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/01380c9b45be474ca0c522f9f5b881ef</t>
+  </si>
+  <si>
     <t>Maximum Number of Added Reactions</t>
   </si>
   <si>
@@ -181,6 +193,9 @@
     <t>{'entropy_weight': 100.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 100.0}</t>
   </si>
   <si>
+    <t>{'entropy_weight': 0.001, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.001}</t>
+  </si>
+  <si>
     <t>Risk Scheduler</t>
   </si>
   <si>
@@ -293,6 +308,9 @@
   </si>
   <si>
     <t>Increased the entropy weight. Gave rise to a slow tail of convergence at the end.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entropy term is now penalizing the whole batch instead of just the topk. This is the correct theoretical way probably. Need to think why exactly. Convergence was very fast. Generative power okay. </t>
   </si>
 </sst>
 </file>
@@ -348,15 +366,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -369,9 +384,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -694,26 +706,28 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:S27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="11" width="22.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="12" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="12" width="24.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="12" width="21.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="12" width="9.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="13" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="12" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="12" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="12" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="14" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="14" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="9" width="22.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="24.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="10" width="21.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="11" width="16.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="10" width="9.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="11" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="10" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="10" width="14.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -762,1390 +776,1542 @@
       <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q2" s="4" t="s">
         <v>33</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="5">
-        <v>5</v>
-      </c>
-      <c r="C3" s="5">
-        <v>5</v>
-      </c>
-      <c r="D3" s="5">
-        <v>5</v>
-      </c>
-      <c r="E3" s="5">
-        <v>5</v>
-      </c>
-      <c r="F3" s="5">
-        <v>5</v>
-      </c>
-      <c r="G3" s="5">
-        <v>5</v>
-      </c>
-      <c r="H3" s="5">
-        <v>5</v>
-      </c>
-      <c r="I3" s="5">
-        <v>5</v>
-      </c>
-      <c r="J3" s="5">
-        <v>5</v>
-      </c>
-      <c r="K3" s="5">
-        <v>5</v>
-      </c>
-      <c r="L3" s="5">
-        <v>5</v>
-      </c>
-      <c r="M3" s="5">
-        <v>5</v>
-      </c>
-      <c r="N3" s="5">
-        <v>5</v>
-      </c>
-      <c r="O3" s="5">
-        <v>5</v>
-      </c>
-      <c r="P3" s="5">
-        <v>5</v>
-      </c>
-      <c r="Q3" s="6">
+        <v>38</v>
+      </c>
+      <c r="B3" s="4">
+        <v>5</v>
+      </c>
+      <c r="C3" s="4">
+        <v>5</v>
+      </c>
+      <c r="D3" s="4">
+        <v>5</v>
+      </c>
+      <c r="E3" s="4">
+        <v>5</v>
+      </c>
+      <c r="F3" s="4">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
+        <v>5</v>
+      </c>
+      <c r="H3" s="4">
+        <v>5</v>
+      </c>
+      <c r="I3" s="4">
+        <v>5</v>
+      </c>
+      <c r="J3" s="4">
+        <v>5</v>
+      </c>
+      <c r="K3" s="4">
+        <v>5</v>
+      </c>
+      <c r="L3" s="4">
+        <v>5</v>
+      </c>
+      <c r="M3" s="4">
+        <v>5</v>
+      </c>
+      <c r="N3" s="4">
+        <v>5</v>
+      </c>
+      <c r="O3" s="4">
+        <v>5</v>
+      </c>
+      <c r="P3" s="4">
+        <v>5</v>
+      </c>
+      <c r="Q3" s="4">
+        <v>5</v>
+      </c>
+      <c r="R3" s="4">
+        <v>5</v>
+      </c>
+      <c r="S3" s="5">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="5">
+        <v>39</v>
+      </c>
+      <c r="B4" s="4">
         <v>3</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>3</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>3</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <v>3</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <v>3</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <v>3</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="4">
         <v>3</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="4">
         <v>3</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="4">
         <v>3</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="4">
         <v>3</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="4">
         <v>3</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="4">
         <v>3</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="4">
         <v>3</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="4">
         <v>3</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="4">
         <v>3</v>
       </c>
-      <c r="Q4" s="6">
+      <c r="Q4" s="4">
+        <v>3</v>
+      </c>
+      <c r="R4" s="4">
+        <v>3</v>
+      </c>
+      <c r="S4" s="5">
         <v>3</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="5">
+        <v>40</v>
+      </c>
+      <c r="B5" s="4">
         <v>2</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>2</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>2</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="4">
         <v>2</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <v>2</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <v>2</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="4">
         <v>2</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="4">
         <v>2</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="4">
         <v>2</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="4">
         <v>2</v>
       </c>
-      <c r="L5" s="5">
+      <c r="L5" s="4">
         <v>2</v>
       </c>
-      <c r="M5" s="5">
+      <c r="M5" s="4">
         <v>2</v>
       </c>
-      <c r="N5" s="5">
+      <c r="N5" s="4">
         <v>2</v>
       </c>
-      <c r="O5" s="5">
+      <c r="O5" s="4">
         <v>2</v>
       </c>
-      <c r="P5" s="5">
+      <c r="P5" s="4">
         <v>2</v>
       </c>
-      <c r="Q5" s="6">
+      <c r="Q5" s="4">
+        <v>2</v>
+      </c>
+      <c r="R5" s="4">
+        <v>2</v>
+      </c>
+      <c r="S5" s="5">
         <v>2</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="5">
+        <v>41</v>
+      </c>
+      <c r="B6" s="4">
         <v>1280</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="4">
         <v>1280</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <v>1280</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="4">
         <v>1280</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <v>1280</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="4">
         <v>1280</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="4">
         <v>2560</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="4">
         <v>2560</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="4">
         <v>2560</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="4">
         <v>2560</v>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="4">
         <v>2560</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="4">
         <v>1280</v>
       </c>
-      <c r="N6" s="5">
+      <c r="N6" s="4">
         <v>1280</v>
       </c>
-      <c r="O6" s="5">
+      <c r="O6" s="4">
         <v>1280</v>
       </c>
-      <c r="P6" s="5">
+      <c r="P6" s="4">
         <v>1280</v>
       </c>
-      <c r="Q6" s="6">
+      <c r="Q6" s="4">
+        <v>1280</v>
+      </c>
+      <c r="R6" s="4">
+        <v>1280</v>
+      </c>
+      <c r="S6" s="5">
         <v>1280</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="7" t="b">
+        <v>42</v>
+      </c>
+      <c r="B7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="C7" s="7" t="b">
+      <c r="C7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="D7" s="7" t="b">
+      <c r="D7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="7" t="b">
+      <c r="E7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="F7" s="7" t="b">
+      <c r="F7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G7" s="7" t="b">
+      <c r="G7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="7" t="b">
+      <c r="H7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="I7" s="7" t="b">
+      <c r="I7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="J7" s="7" t="b">
+      <c r="J7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="K7" s="7" t="b">
+      <c r="K7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="L7" s="7" t="b">
+      <c r="L7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="M7" s="7" t="b">
+      <c r="M7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="N7" s="7" t="b">
+      <c r="N7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="O7" s="7" t="b">
+      <c r="O7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="P7" s="8" t="b">
+      <c r="P7" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="Q7" s="4" t="b">
+      <c r="Q7" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="R7" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" s="3" t="b">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="9">
+        <v>43</v>
+      </c>
+      <c r="B8" s="7">
         <v>0.0001</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="7">
         <v>0.0001</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="J8" s="9">
+      <c r="J8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="M8" s="9">
+      <c r="M8" s="7">
         <v>0.0001</v>
       </c>
-      <c r="N8" s="9">
+      <c r="N8" s="7">
         <v>0.0001</v>
       </c>
-      <c r="O8" s="9">
+      <c r="O8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="P8" s="9">
+      <c r="P8" s="7">
         <v>0.00001</v>
       </c>
-      <c r="Q8" s="10">
+      <c r="Q8" s="7">
         <v>0.00001</v>
+      </c>
+      <c r="R8" s="7">
+        <v>0.0001</v>
+      </c>
+      <c r="S8" s="8">
+        <v>0.0001</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="5">
+        <v>44</v>
+      </c>
+      <c r="B9" s="4">
         <v>300</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="4">
         <v>300</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="4">
         <v>300</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="4">
         <v>300</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="4">
         <v>300</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <v>500</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="4">
         <v>500</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="4">
         <v>500</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="4">
         <v>500</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="4">
         <v>500</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="4">
         <v>300</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="4">
         <v>300</v>
       </c>
-      <c r="N9" s="5">
+      <c r="N9" s="4">
         <v>300</v>
       </c>
-      <c r="O9" s="5">
+      <c r="O9" s="4">
         <v>500</v>
       </c>
-      <c r="P9" s="5">
+      <c r="P9" s="4">
         <v>500</v>
       </c>
-      <c r="Q9" s="6">
+      <c r="Q9" s="4">
         <v>500</v>
+      </c>
+      <c r="R9" s="4">
+        <v>300</v>
+      </c>
+      <c r="S9" s="5">
+        <v>300</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="5">
-        <v>5</v>
-      </c>
-      <c r="C10" s="5">
-        <v>5</v>
-      </c>
-      <c r="D10" s="5">
-        <v>5</v>
-      </c>
-      <c r="E10" s="5">
-        <v>5</v>
-      </c>
-      <c r="F10" s="5">
-        <v>5</v>
-      </c>
-      <c r="G10" s="5">
-        <v>5</v>
-      </c>
-      <c r="H10" s="5">
-        <v>5</v>
-      </c>
-      <c r="I10" s="5">
-        <v>5</v>
-      </c>
-      <c r="J10" s="5">
-        <v>5</v>
-      </c>
-      <c r="K10" s="5">
-        <v>5</v>
-      </c>
-      <c r="L10" s="5">
-        <v>5</v>
-      </c>
-      <c r="M10" s="5">
-        <v>5</v>
-      </c>
-      <c r="N10" s="5">
-        <v>5</v>
-      </c>
-      <c r="O10" s="5">
-        <v>5</v>
-      </c>
-      <c r="P10" s="5">
-        <v>5</v>
-      </c>
-      <c r="Q10" s="6">
+        <v>45</v>
+      </c>
+      <c r="B10" s="4">
+        <v>5</v>
+      </c>
+      <c r="C10" s="4">
+        <v>5</v>
+      </c>
+      <c r="D10" s="4">
+        <v>5</v>
+      </c>
+      <c r="E10" s="4">
+        <v>5</v>
+      </c>
+      <c r="F10" s="4">
+        <v>5</v>
+      </c>
+      <c r="G10" s="4">
+        <v>5</v>
+      </c>
+      <c r="H10" s="4">
+        <v>5</v>
+      </c>
+      <c r="I10" s="4">
+        <v>5</v>
+      </c>
+      <c r="J10" s="4">
+        <v>5</v>
+      </c>
+      <c r="K10" s="4">
+        <v>5</v>
+      </c>
+      <c r="L10" s="4">
+        <v>5</v>
+      </c>
+      <c r="M10" s="4">
+        <v>5</v>
+      </c>
+      <c r="N10" s="4">
+        <v>5</v>
+      </c>
+      <c r="O10" s="4">
+        <v>5</v>
+      </c>
+      <c r="P10" s="4">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="4">
+        <v>5</v>
+      </c>
+      <c r="R10" s="4">
+        <v>5</v>
+      </c>
+      <c r="S10" s="5">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B11" s="5">
+        <v>46</v>
+      </c>
+      <c r="B11" s="4">
         <v>1024</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="4">
         <v>1024</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="4">
         <v>1024</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="4">
         <v>1024</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="4">
         <v>1024</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="4">
         <v>1024</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="4">
         <v>1024</v>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="4">
         <v>1024</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="4">
         <v>1024</v>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="4">
         <v>1024</v>
       </c>
-      <c r="L11" s="5">
+      <c r="L11" s="4">
         <v>1024</v>
       </c>
-      <c r="M11" s="5">
+      <c r="M11" s="4">
         <v>1024</v>
       </c>
-      <c r="N11" s="5">
+      <c r="N11" s="4">
         <v>1024</v>
       </c>
-      <c r="O11" s="5">
+      <c r="O11" s="4">
         <v>1024</v>
       </c>
-      <c r="P11" s="5">
+      <c r="P11" s="4">
         <v>1024</v>
       </c>
-      <c r="Q11" s="6">
+      <c r="Q11" s="4">
+        <v>1024</v>
+      </c>
+      <c r="R11" s="4">
+        <v>1024</v>
+      </c>
+      <c r="S11" s="5">
         <v>1024</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B12" s="5">
+        <v>47</v>
+      </c>
+      <c r="B12" s="4">
         <v>10240</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="4">
         <v>10240</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="4">
         <v>10240</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="4">
         <v>10240</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="4">
         <v>10240</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="4">
         <v>10240</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="4">
         <v>10240</v>
       </c>
-      <c r="I12" s="5">
+      <c r="I12" s="4">
         <v>10240</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="4">
         <v>10240</v>
       </c>
-      <c r="K12" s="5">
+      <c r="K12" s="4">
         <v>10240</v>
       </c>
-      <c r="L12" s="5">
+      <c r="L12" s="4">
         <v>10240</v>
       </c>
-      <c r="M12" s="5">
+      <c r="M12" s="4">
         <v>10240</v>
       </c>
-      <c r="N12" s="5">
+      <c r="N12" s="4">
         <v>10240</v>
       </c>
-      <c r="O12" s="5">
+      <c r="O12" s="4">
         <v>10240</v>
       </c>
-      <c r="P12" s="5">
+      <c r="P12" s="4">
         <v>10240</v>
       </c>
-      <c r="Q12" s="6">
+      <c r="Q12" s="4">
+        <v>10240</v>
+      </c>
+      <c r="R12" s="4">
+        <v>10240</v>
+      </c>
+      <c r="S12" s="5">
         <v>10240</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="5">
+        <v>48</v>
+      </c>
+      <c r="B13" s="4">
         <v>128</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="4">
         <v>128</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="4">
         <v>128</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="4">
         <v>128</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="4">
         <v>128</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="4">
         <v>128</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="4">
         <v>128</v>
       </c>
-      <c r="I13" s="5">
+      <c r="I13" s="4">
         <v>128</v>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="4">
         <v>128</v>
       </c>
-      <c r="K13" s="5">
+      <c r="K13" s="4">
         <v>128</v>
       </c>
-      <c r="L13" s="5">
+      <c r="L13" s="4">
         <v>128</v>
       </c>
-      <c r="M13" s="5">
+      <c r="M13" s="4">
         <v>128</v>
       </c>
-      <c r="N13" s="5">
+      <c r="N13" s="4">
         <v>128</v>
       </c>
-      <c r="O13" s="5">
+      <c r="O13" s="4">
         <v>128</v>
       </c>
-      <c r="P13" s="5">
+      <c r="P13" s="4">
         <v>128</v>
       </c>
-      <c r="Q13" s="6">
+      <c r="Q13" s="4">
+        <v>128</v>
+      </c>
+      <c r="R13" s="4">
+        <v>128</v>
+      </c>
+      <c r="S13" s="5">
         <v>128</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="P14" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q14" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="S14" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="P15" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q15" s="4" t="s">
-        <v>57</v>
+        <v>63</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="S15" s="3" t="s">
+        <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B16" s="5">
-        <v>1</v>
-      </c>
-      <c r="C16" s="5">
-        <v>1</v>
-      </c>
-      <c r="D16" s="5">
-        <v>1</v>
-      </c>
-      <c r="E16" s="5">
-        <v>1</v>
-      </c>
-      <c r="F16" s="5">
-        <v>1</v>
-      </c>
-      <c r="G16" s="5">
-        <v>1</v>
-      </c>
-      <c r="H16" s="5">
-        <v>1</v>
-      </c>
-      <c r="I16" s="5">
-        <v>1</v>
-      </c>
-      <c r="J16" s="5">
-        <v>1</v>
-      </c>
-      <c r="K16" s="5">
-        <v>1</v>
-      </c>
-      <c r="L16" s="5">
-        <v>1</v>
-      </c>
-      <c r="M16" s="5">
-        <v>1</v>
-      </c>
-      <c r="N16" s="5">
-        <v>1</v>
-      </c>
-      <c r="O16" s="5">
-        <v>1</v>
-      </c>
-      <c r="P16" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q16" s="6">
+        <v>64</v>
+      </c>
+      <c r="B16" s="4">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4">
+        <v>1</v>
+      </c>
+      <c r="D16" s="4">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4">
+        <v>1</v>
+      </c>
+      <c r="F16" s="4">
+        <v>1</v>
+      </c>
+      <c r="G16" s="4">
+        <v>1</v>
+      </c>
+      <c r="H16" s="4">
+        <v>1</v>
+      </c>
+      <c r="I16" s="4">
+        <v>1</v>
+      </c>
+      <c r="J16" s="4">
+        <v>1</v>
+      </c>
+      <c r="K16" s="4">
+        <v>1</v>
+      </c>
+      <c r="L16" s="4">
+        <v>1</v>
+      </c>
+      <c r="M16" s="4">
+        <v>1</v>
+      </c>
+      <c r="N16" s="4">
+        <v>1</v>
+      </c>
+      <c r="O16" s="4">
+        <v>1</v>
+      </c>
+      <c r="P16" s="4">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="4">
+        <v>1</v>
+      </c>
+      <c r="R16" s="4">
+        <v>1</v>
+      </c>
+      <c r="S16" s="5">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B17" s="5">
-        <v>1</v>
-      </c>
-      <c r="C17" s="5">
-        <v>1</v>
-      </c>
-      <c r="D17" s="5">
-        <v>1</v>
-      </c>
-      <c r="E17" s="5">
-        <v>1</v>
-      </c>
-      <c r="F17" s="5">
-        <v>1</v>
-      </c>
-      <c r="G17" s="5">
-        <v>1</v>
-      </c>
-      <c r="H17" s="5">
-        <v>1</v>
-      </c>
-      <c r="I17" s="5">
-        <v>1</v>
-      </c>
-      <c r="J17" s="5">
-        <v>1</v>
-      </c>
-      <c r="K17" s="5">
-        <v>1</v>
-      </c>
-      <c r="L17" s="5">
-        <v>1</v>
-      </c>
-      <c r="M17" s="5">
-        <v>1</v>
-      </c>
-      <c r="N17" s="5">
-        <v>1</v>
-      </c>
-      <c r="O17" s="5">
-        <v>1</v>
-      </c>
-      <c r="P17" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q17" s="6">
+        <v>65</v>
+      </c>
+      <c r="B17" s="4">
+        <v>1</v>
+      </c>
+      <c r="C17" s="4">
+        <v>1</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1</v>
+      </c>
+      <c r="E17" s="4">
+        <v>1</v>
+      </c>
+      <c r="F17" s="4">
+        <v>1</v>
+      </c>
+      <c r="G17" s="4">
+        <v>1</v>
+      </c>
+      <c r="H17" s="4">
+        <v>1</v>
+      </c>
+      <c r="I17" s="4">
+        <v>1</v>
+      </c>
+      <c r="J17" s="4">
+        <v>1</v>
+      </c>
+      <c r="K17" s="4">
+        <v>1</v>
+      </c>
+      <c r="L17" s="4">
+        <v>1</v>
+      </c>
+      <c r="M17" s="4">
+        <v>1</v>
+      </c>
+      <c r="N17" s="4">
+        <v>1</v>
+      </c>
+      <c r="O17" s="4">
+        <v>1</v>
+      </c>
+      <c r="P17" s="4">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="4">
+        <v>1</v>
+      </c>
+      <c r="R17" s="4">
+        <v>1</v>
+      </c>
+      <c r="S17" s="5">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B18" s="5">
+        <v>66</v>
+      </c>
+      <c r="B18" s="4">
         <v>200</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="4">
         <v>200</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="4">
         <v>200</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="4">
         <v>200</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="4">
         <v>200</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="4">
         <v>200</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="4">
         <v>200</v>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="4">
         <v>200</v>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="4">
         <v>200</v>
       </c>
-      <c r="K18" s="5">
+      <c r="K18" s="4">
         <v>200</v>
       </c>
-      <c r="L18" s="5">
+      <c r="L18" s="4">
         <v>200</v>
       </c>
-      <c r="M18" s="5">
+      <c r="M18" s="4">
         <v>200</v>
       </c>
-      <c r="N18" s="5">
+      <c r="N18" s="4">
         <v>200</v>
       </c>
-      <c r="O18" s="5">
+      <c r="O18" s="4">
         <v>200</v>
       </c>
-      <c r="P18" s="5">
+      <c r="P18" s="4">
         <v>200</v>
       </c>
-      <c r="Q18" s="6">
+      <c r="Q18" s="4">
+        <v>200</v>
+      </c>
+      <c r="R18" s="4">
+        <v>200</v>
+      </c>
+      <c r="S18" s="5">
         <v>200</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" s="5">
+        <v>67</v>
+      </c>
+      <c r="B19" s="4">
         <v>1000</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="4">
         <v>1000</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="4">
         <v>1000</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="4">
         <v>1000</v>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="4">
         <v>1000</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="4">
         <v>1000</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="4">
         <v>1000</v>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="4">
         <v>1000</v>
       </c>
-      <c r="J19" s="5">
+      <c r="J19" s="4">
         <v>1000</v>
       </c>
-      <c r="K19" s="5">
+      <c r="K19" s="4">
         <v>1000</v>
       </c>
-      <c r="L19" s="5">
+      <c r="L19" s="4">
         <v>1000</v>
       </c>
-      <c r="M19" s="5">
+      <c r="M19" s="4">
         <v>1000</v>
       </c>
-      <c r="N19" s="5">
+      <c r="N19" s="4">
         <v>1000</v>
       </c>
-      <c r="O19" s="5">
+      <c r="O19" s="4">
         <v>1000</v>
       </c>
-      <c r="P19" s="5">
+      <c r="P19" s="4">
         <v>1000</v>
       </c>
-      <c r="Q19" s="6">
+      <c r="Q19" s="4">
+        <v>1000</v>
+      </c>
+      <c r="R19" s="4">
+        <v>1000</v>
+      </c>
+      <c r="S19" s="5">
         <v>1000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B20" s="5">
-        <v>1</v>
-      </c>
-      <c r="C20" s="5">
-        <v>1</v>
-      </c>
-      <c r="D20" s="5">
-        <v>1</v>
-      </c>
-      <c r="E20" s="5">
-        <v>1</v>
-      </c>
-      <c r="F20" s="5">
-        <v>1</v>
-      </c>
-      <c r="G20" s="5">
-        <v>1</v>
-      </c>
-      <c r="H20" s="5">
-        <v>1</v>
-      </c>
-      <c r="I20" s="5">
-        <v>1</v>
-      </c>
-      <c r="J20" s="5">
-        <v>1</v>
-      </c>
-      <c r="K20" s="5">
-        <v>1</v>
-      </c>
-      <c r="L20" s="5">
-        <v>1</v>
-      </c>
-      <c r="M20" s="5">
-        <v>1</v>
-      </c>
-      <c r="N20" s="5">
-        <v>1</v>
-      </c>
-      <c r="O20" s="5">
-        <v>1</v>
-      </c>
-      <c r="P20" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="6">
+        <v>68</v>
+      </c>
+      <c r="B20" s="4">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4">
+        <v>1</v>
+      </c>
+      <c r="D20" s="4">
+        <v>1</v>
+      </c>
+      <c r="E20" s="4">
+        <v>1</v>
+      </c>
+      <c r="F20" s="4">
+        <v>1</v>
+      </c>
+      <c r="G20" s="4">
+        <v>1</v>
+      </c>
+      <c r="H20" s="4">
+        <v>1</v>
+      </c>
+      <c r="I20" s="4">
+        <v>1</v>
+      </c>
+      <c r="J20" s="4">
+        <v>1</v>
+      </c>
+      <c r="K20" s="4">
+        <v>1</v>
+      </c>
+      <c r="L20" s="4">
+        <v>1</v>
+      </c>
+      <c r="M20" s="4">
+        <v>1</v>
+      </c>
+      <c r="N20" s="4">
+        <v>1</v>
+      </c>
+      <c r="O20" s="4">
+        <v>1</v>
+      </c>
+      <c r="P20" s="4">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="4">
+        <v>1</v>
+      </c>
+      <c r="R20" s="4">
+        <v>1</v>
+      </c>
+      <c r="S20" s="5">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B21" s="5">
+        <v>69</v>
+      </c>
+      <c r="B21" s="4">
         <v>9</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="4">
         <v>9</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="4">
         <v>9</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="4">
         <v>9</v>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="4">
         <v>9</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="4">
         <v>9</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="4">
         <v>9</v>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="4">
         <v>9</v>
       </c>
-      <c r="J21" s="5">
+      <c r="J21" s="4">
         <v>9</v>
       </c>
-      <c r="K21" s="5">
+      <c r="K21" s="4">
         <v>9</v>
       </c>
-      <c r="L21" s="5">
+      <c r="L21" s="4">
         <v>9</v>
       </c>
-      <c r="M21" s="5">
+      <c r="M21" s="4">
         <v>9</v>
       </c>
-      <c r="N21" s="5">
+      <c r="N21" s="4">
         <v>9</v>
       </c>
-      <c r="O21" s="5">
+      <c r="O21" s="4">
         <v>9</v>
       </c>
-      <c r="P21" s="5">
+      <c r="P21" s="4">
         <v>9</v>
       </c>
-      <c r="Q21" s="6">
+      <c r="Q21" s="4">
+        <v>9</v>
+      </c>
+      <c r="R21" s="4">
+        <v>9</v>
+      </c>
+      <c r="S21" s="5">
         <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="P22" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q22" s="4" t="s">
-        <v>68</v>
+        <v>73</v>
+      </c>
+      <c r="P22" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q22" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="S22" s="3" t="s">
+        <v>73</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="J23" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="L23" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="P23" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q23" s="4" t="s">
-        <v>71</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="P23" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q23" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="R23" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="S23" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>70</v>
+        <v>75</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>75</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="J24" s="5" t="s">
-        <v>71</v>
+        <v>75</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="L24" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="P24" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q24" s="4" t="s">
-        <v>73</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="P24" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q24" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="R24" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="S24" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>71</v>
+        <v>75</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="L25" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="O25" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="P25" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q25" s="4" t="s">
-        <v>71</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="P25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="R25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="S25" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>71</v>
+        <v>75</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="L26" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="O26" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="P26" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q26" s="4" t="s">
-        <v>70</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="P26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="R26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="S26" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="J27" s="5" t="s">
-        <v>85</v>
+        <v>89</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="L27" s="5" t="s">
-        <v>87</v>
+        <v>91</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>92</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="O27" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="P27" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="Q27" s="4" t="s">
-        <v>92</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="P27" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q27" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="R27" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="S27" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fixed bug in renderer for closing the figures.
</commit_message>
<xml_diff>
--- a/apps/RPA_3species_5rxns_REINFORCE/RPA_3species_5rxns_MAK_REINFORCE.xlsx
+++ b/apps/RPA_3species_5rxns_REINFORCE/RPA_3species_5rxns_MAK_REINFORCE.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="100">
   <si>
     <t>Timestamp</t>
   </si>
@@ -70,7 +70,7 @@
     <t>2025-11-07 12:20:24</t>
   </si>
   <si>
-    <t>2025-11-07 15:10:13</t>
+    <t>2025-11-07 16:38:38</t>
   </si>
   <si>
     <t>URL</t>
@@ -127,7 +127,7 @@
     <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/cb4a2ecf6dc447df8caee14bdedbe11e</t>
   </si>
   <si>
-    <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/01380c9b45be474ca0c522f9f5b881ef</t>
+    <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/472a8c7424f44cbfada965f2b2b7c949</t>
   </si>
   <si>
     <t>Maximum Number of Added Reactions</t>
@@ -194,6 +194,9 @@
   </si>
   <si>
     <t>{'entropy_weight': 0.001, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.001}</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.005, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.005}</t>
   </si>
   <si>
     <t>Risk Scheduler</t>
@@ -1553,71 +1556,71 @@
         <v>59</v>
       </c>
       <c r="S14" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="R15" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="S15" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="O15" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P15" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q15" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="S15" s="3" t="s">
-        <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B16" s="4">
         <v>1</v>
@@ -1676,7 +1679,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B17" s="4">
         <v>1</v>
@@ -1735,7 +1738,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B18" s="4">
         <v>200</v>
@@ -1794,7 +1797,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B19" s="4">
         <v>1000</v>
@@ -1853,7 +1856,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B20" s="4">
         <v>1</v>
@@ -1912,7 +1915,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B21" s="4">
         <v>9</v>
@@ -1971,345 +1974,345 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q22" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R22" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L23" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="R23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="S23" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q24" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="R24" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="S24" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L25" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="P25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="R25" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="S25" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="R26" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="S26" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="O27" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P27" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="Q27" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="R27" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="S27" s="3"/>
     </row>

</xml_diff>